<commit_message>
fix(browser): validate the shared Engine contract before launch
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -13952,7 +13952,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="E169" s="3" t="str">
-        <x:v>Runtime admits page and engine; unavailable engine/network is explicit rather than a blank success.</x:v>
+        <x:v>Runtime admits a compatible Engine before page, profile or stream effects. A version or capability mismatch has a typed, actionable error.</x:v>
       </x:c>
       <x:c r="F169" s="12" t="str">
         <x:v>Earlier foreground runs found intermittent startup and navigation failures. E-108 adds a current cold launch: the macOS VM path reached Ready in 38.5 seconds, then Home Close removed the VM supervisor, VZ supervisor, and TURN process. The older intermittent finding remains open until repeated navigation and restart acceptance passes.</x:v>
@@ -13961,14 +13961,15 @@
         <x:v>controlled-network</x:v>
       </x:c>
       <x:c r="H169" s="3" t="str">
-        <x:v>implemented-source</x:v>
+        <x:v>Shared Engine contract and pre-effect compatibility route tests pass. Installed acceptance pending.</x:v>
       </x:c>
       <x:c r="I169" s="3" t="str">
         <x:v>Address; Navigate/Enter; Loading/status</x:v>
       </x:c>
       <x:c r="J169" s="3" t="str">
-        <x:v>1. Open Browser
-2. Use approved harmless URL</x:v>
+        <x:v>1. Open an approved harmless URL
+2. Use an incompatible Engine fixture
+3. Verify typed rejection before page/profile/stream allocation</x:v>
       </x:c>
       <x:c r="K169" s="3" t="str">
         <x:v>Approved public page; Running Browser substrate</x:v>
@@ -14084,7 +14085,7 @@
         <x:v>Partially observed</x:v>
       </x:c>
       <x:c r="E171" s="3" t="str">
-        <x:v>Runtime selects engine/Exit from projected offers; capsule receives no peer/route authority.</x:v>
+        <x:v>Runtime selects from admitted Engine/Exit offers. Automatic Engine selection meets display/isolation requirements. Explicit selection preserves operator intent.</x:v>
       </x:c>
       <x:c r="F171" s="12" t="str">
         <x:v>Settings exposes the local MicroVM engine and This device Exit; disabled during load and enabled after Ready. Selections/configuration preserved; controlled remote-service switch lacks a peer fixture.</x:v>
@@ -14093,14 +14094,16 @@
         <x:v>controlled-service</x:v>
       </x:c>
       <x:c r="H171" s="3" t="str">
-        <x:v>implemented-source</x:v>
+        <x:v>Shared inventory validates versions and capabilities. Automatic and explicit selection tests pass. Remote installed proof pending.</x:v>
       </x:c>
       <x:c r="I171" s="3" t="str">
         <x:v>Settings; Browser Engine; Exit</x:v>
       </x:c>
       <x:c r="J171" s="3" t="str">
         <x:v>1. Inspect local/remote choices
-2. Change only controlled available service</x:v>
+2. Select a controlled service
+3. Test incompatible default and explicit Engine
+4. Verify approved compatible choice or typed rejection</x:v>
       </x:c>
       <x:c r="K171" s="3" t="str">
         <x:v>Operator-approved service selection</x:v>

</xml_diff>

<commit_message>
fix(browser): check viewer capabilities before replacing a page
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -13952,7 +13952,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="E169" s="3" t="str">
-        <x:v>Runtime admits a compatible Engine before page, profile or stream effects. A version or capability mismatch has a typed, actionable error.</x:v>
+        <x:v>Viewer eligibility is checked before page replacement. Runtime admits a compatible Engine before page, profile or stream effects. Both report typed compatibility errors.</x:v>
       </x:c>
       <x:c r="F169" s="12" t="str">
         <x:v>Earlier foreground runs found intermittent startup and navigation failures. E-108 adds a current cold launch: the macOS VM path reached Ready in 38.5 seconds, then Home Close removed the VM supervisor, VZ supervisor, and TURN process. The older intermittent finding remains open until repeated navigation and restart acceptance passes.</x:v>
@@ -13961,7 +13961,7 @@
         <x:v>controlled-network</x:v>
       </x:c>
       <x:c r="H169" s="3" t="str">
-        <x:v>Shared Engine contract and pre-effect compatibility route tests pass. Installed acceptance pending.</x:v>
+        <x:v>Engine compatibility and viewer preflight tests pass, including preservation of an existing page on viewer denial. Installed acceptance pending.</x:v>
       </x:c>
       <x:c r="I169" s="3" t="str">
         <x:v>Address; Navigate/Enter; Loading/status</x:v>
@@ -13969,7 +13969,8 @@
       <x:c r="J169" s="3" t="str">
         <x:v>1. Open an approved harmless URL
 2. Use an incompatible Engine fixture
-3. Verify typed rejection before page/profile/stream allocation</x:v>
+3. Verify typed rejection before page/profile/stream allocation
+4. Disable viewer WebRTC in a controlled fixture; verify typed rejection and preservation of an existing page</x:v>
       </x:c>
       <x:c r="K169" s="3" t="str">
         <x:v>Approved public page; Running Browser substrate</x:v>

</xml_diff>

<commit_message>
docs(browser): record installed viewer and operator proof
</commit_message>
<xml_diff>
--- a/docs/audits/ElastOS-Home-Journey-Audit.xlsx
+++ b/docs/audits/ElastOS-Home-Journey-Audit.xlsx
@@ -3462,7 +3462,7 @@
         <x:v>Blocked prerequisite</x:v>
       </x:c>
       <x:c r="E8" s="3" t="str">
-        <x:v>Valid passkey opens that principal's shell; cancellation leaves Home locked.</x:v>
+        <x:v>People and agents can find the passkey control. A valid passkey opens the same principal's shell; cancellation leaves Home locked.</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
         <x:v>Brave resumes the existing authenticated session. A fresh passkey sign-in was not forced because it would disturb the current session.</x:v>
@@ -3471,15 +3471,16 @@
         <x:v>controlled-identity</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>implemented-source</x:v>
+        <x:v>Isolated B01 Brave sign-in passed. Full Home qualification remains open.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
         <x:v>Use passkey; Account picker</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
         <x:v>1. Open signed-out Home
-2. Choose existing account
-3. Use passkey</x:v>
+2. Find the passkey control by its accessible role and label
+3. Use passkey
+4. Verify the same principal's shell</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>Existing disposable test account</x:v>
@@ -13961,7 +13962,7 @@
         <x:v>controlled-network</x:v>
       </x:c>
       <x:c r="H169" s="3" t="str">
-        <x:v>Engine compatibility and viewer preflight tests pass, including preservation of an existing page on viewer denial. Installed acceptance pending.</x:v>
+        <x:v>Installed Brave viewer denial passed: zero Engine requests, zero Runtime sessions, clean window close. Engine media proof remains open.</x:v>
       </x:c>
       <x:c r="I169" s="3" t="str">
         <x:v>Address; Navigate/Enter; Loading/status</x:v>

</xml_diff>